<commit_message>
moved sequelize code to its own folder
</commit_message>
<xml_diff>
--- a/Statistics/Early results.xlsx
+++ b/Statistics/Early results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eveda-my.sharepoint.com/personal/erik_eveda_se/Documents/School Work/Examensarbete/Typescript/Petclinic/Statistics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{17E96A0E-954F-45CD-A560-4394AB74B44A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="213" documentId="8_{17E96A0E-954F-45CD-A560-4394AB74B44A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1AB245A9-C208-4099-A20F-C04A75BA8FF5}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{58876018-79A1-4442-99DF-21D6448809B6}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="20">
   <si>
     <t>Mean</t>
   </si>
@@ -86,10 +86,16 @@
     <t>Simple select</t>
   </si>
   <si>
-    <t>AllOwners</t>
+    <t>Mean Respons Time</t>
   </si>
   <si>
-    <t>Mean Respons Time</t>
+    <t>AllOwners delay</t>
+  </si>
+  <si>
+    <t>Simple select delay</t>
+  </si>
+  <si>
+    <t>All Owners</t>
   </si>
 </sst>
 </file>
@@ -160,14 +166,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -220,7 +230,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="sv-SE"/>
-              <a:t>All Owners</a:t>
+              <a:t>All Owners Delay</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -287,28 +297,28 @@
           <c:invertIfNegative val="0"/>
           <c:errBars>
             <c:errBarType val="both"/>
-            <c:errValType val="stdErr"/>
+            <c:errValType val="cust"/>
             <c:noEndCap val="0"/>
             <c:plus>
               <c:numRef>
-                <c:f>Responstime!$G$9</c:f>
+                <c:f>Responstime!$G$6</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="1"/>
                   <c:pt idx="0">
-                    <c:v>0.5</c:v>
+                    <c:v>0.16666666666666666</c:v>
                   </c:pt>
                 </c:numCache>
               </c:numRef>
             </c:plus>
             <c:minus>
               <c:numRef>
-                <c:f>Responstime!$G$9</c:f>
+                <c:f>Responstime!$G$6</c:f>
                 <c:numCache>
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="1"/>
                   <c:pt idx="0">
-                    <c:v>0.5</c:v>
+                    <c:v>0.16666666666666666</c:v>
                   </c:pt>
                 </c:numCache>
               </c:numRef>
@@ -382,8 +392,32 @@
           <c:invertIfNegative val="0"/>
           <c:errBars>
             <c:errBarType val="both"/>
-            <c:errValType val="stdErr"/>
+            <c:errValType val="cust"/>
             <c:noEndCap val="0"/>
+            <c:plus>
+              <c:numRef>
+                <c:f>Responstime!$I$6</c:f>
+                <c:numCache>
+                  <c:formatCode>General</c:formatCode>
+                  <c:ptCount val="1"/>
+                  <c:pt idx="0">
+                    <c:v>0.16666666666666666</c:v>
+                  </c:pt>
+                </c:numCache>
+              </c:numRef>
+            </c:plus>
+            <c:minus>
+              <c:numRef>
+                <c:f>Responstime!$I$6</c:f>
+                <c:numCache>
+                  <c:formatCode>General</c:formatCode>
+                  <c:ptCount val="1"/>
+                  <c:pt idx="0">
+                    <c:v>0.16666666666666666</c:v>
+                  </c:pt>
+                </c:numCache>
+              </c:numRef>
+            </c:minus>
             <c:spPr>
               <a:noFill/>
               <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
@@ -668,11 +702,11 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="sv-SE"/>
-              <a:t>All Pets From</a:t>
+              <a:t>Simple Select </a:t>
             </a:r>
             <a:r>
               <a:rPr lang="sv-SE" baseline="0"/>
-              <a:t> City</a:t>
+              <a:t>Delay</a:t>
             </a:r>
             <a:endParaRPr lang="sv-SE"/>
           </a:p>
@@ -738,6 +772,48 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:errBars>
+            <c:errBarType val="both"/>
+            <c:errValType val="cust"/>
+            <c:noEndCap val="0"/>
+            <c:plus>
+              <c:numRef>
+                <c:f>Responstime!$G$25</c:f>
+                <c:numCache>
+                  <c:formatCode>General</c:formatCode>
+                  <c:ptCount val="1"/>
+                  <c:pt idx="0">
+                    <c:v>0.24944382578492943</c:v>
+                  </c:pt>
+                </c:numCache>
+              </c:numRef>
+            </c:plus>
+            <c:minus>
+              <c:numRef>
+                <c:f>Responstime!$G$25</c:f>
+                <c:numCache>
+                  <c:formatCode>General</c:formatCode>
+                  <c:ptCount val="1"/>
+                  <c:pt idx="0">
+                    <c:v>0.24944382578492943</c:v>
+                  </c:pt>
+                </c:numCache>
+              </c:numRef>
+            </c:minus>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:errBars>
           <c:cat>
             <c:strRef>
               <c:f>Responstime!$U$3</c:f>
@@ -791,6 +867,48 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:errBars>
+            <c:errBarType val="both"/>
+            <c:errValType val="cust"/>
+            <c:noEndCap val="0"/>
+            <c:plus>
+              <c:numRef>
+                <c:f>Responstime!$I$25</c:f>
+                <c:numCache>
+                  <c:formatCode>General</c:formatCode>
+                  <c:ptCount val="1"/>
+                  <c:pt idx="0">
+                    <c:v>9.9999999999999992E-2</c:v>
+                  </c:pt>
+                </c:numCache>
+              </c:numRef>
+            </c:plus>
+            <c:minus>
+              <c:numRef>
+                <c:f>Responstime!$I$25</c:f>
+                <c:numCache>
+                  <c:formatCode>General</c:formatCode>
+                  <c:ptCount val="1"/>
+                  <c:pt idx="0">
+                    <c:v>9.9999999999999992E-2</c:v>
+                  </c:pt>
+                </c:numCache>
+              </c:numRef>
+            </c:minus>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:errBars>
           <c:cat>
             <c:strRef>
               <c:f>Responstime!$U$3</c:f>
@@ -1023,6 +1141,951 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="sv-SE"/>
+              <a:t>All</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="sv-SE" baseline="0"/>
+              <a:t> pets from city (Advanced)</a:t>
+            </a:r>
+            <a:endParaRPr lang="sv-SE"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="sv-SE"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Responstime!$F$43</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Sequlize</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:errBars>
+            <c:errBarType val="both"/>
+            <c:errValType val="cust"/>
+            <c:noEndCap val="0"/>
+            <c:plus>
+              <c:numRef>
+                <c:f>Responstime!$G$46</c:f>
+                <c:numCache>
+                  <c:formatCode>General</c:formatCode>
+                  <c:ptCount val="1"/>
+                  <c:pt idx="0">
+                    <c:v>0.17950549357115031</c:v>
+                  </c:pt>
+                </c:numCache>
+              </c:numRef>
+            </c:plus>
+            <c:minus>
+              <c:numRef>
+                <c:f>Responstime!$G$46</c:f>
+                <c:numCache>
+                  <c:formatCode>General</c:formatCode>
+                  <c:ptCount val="1"/>
+                  <c:pt idx="0">
+                    <c:v>0.17950549357115031</c:v>
+                  </c:pt>
+                </c:numCache>
+              </c:numRef>
+            </c:minus>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:errBars>
+          <c:cat>
+            <c:strRef>
+              <c:f>Responstime!$U$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Mean Respons Time</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Responstime!$G$45</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>4.0999999999999996</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-C905-4BAD-8B75-F400E22ED858}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Responstime!$H$43</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Pure</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:errBars>
+            <c:errBarType val="both"/>
+            <c:errValType val="cust"/>
+            <c:noEndCap val="0"/>
+            <c:plus>
+              <c:numRef>
+                <c:f>Responstime!$I$46</c:f>
+                <c:numCache>
+                  <c:formatCode>General</c:formatCode>
+                  <c:ptCount val="1"/>
+                  <c:pt idx="0">
+                    <c:v>9.9999999999999992E-2</c:v>
+                  </c:pt>
+                </c:numCache>
+              </c:numRef>
+            </c:plus>
+            <c:minus>
+              <c:numRef>
+                <c:f>Responstime!$I$46</c:f>
+                <c:numCache>
+                  <c:formatCode>General</c:formatCode>
+                  <c:ptCount val="1"/>
+                  <c:pt idx="0">
+                    <c:v>9.9999999999999992E-2</c:v>
+                  </c:pt>
+                </c:numCache>
+              </c:numRef>
+            </c:minus>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:errBars>
+          <c:cat>
+            <c:strRef>
+              <c:f>Responstime!$U$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Mean Respons Time</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Responstime!$I$45</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>3.1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-C905-4BAD-8B75-F400E22ED858}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1087496143"/>
+        <c:axId val="1087507663"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1087496143"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="sv-SE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1087507663"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1087507663"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="sv-SE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1087496143"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="sv-SE"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="sv-SE"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="sv-SE"/>
+              <a:t>All Owners (Simple)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="sv-SE"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Responstime!$F$63</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Sequlize</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:errBars>
+            <c:errBarType val="both"/>
+            <c:errValType val="cust"/>
+            <c:noEndCap val="0"/>
+            <c:plus>
+              <c:numRef>
+                <c:f>Responstime!$G$66</c:f>
+                <c:numCache>
+                  <c:formatCode>General</c:formatCode>
+                  <c:ptCount val="1"/>
+                  <c:pt idx="0">
+                    <c:v>0.16329931618554538</c:v>
+                  </c:pt>
+                </c:numCache>
+              </c:numRef>
+            </c:plus>
+            <c:minus>
+              <c:numRef>
+                <c:f>Responstime!$G$66</c:f>
+                <c:numCache>
+                  <c:formatCode>General</c:formatCode>
+                  <c:ptCount val="1"/>
+                  <c:pt idx="0">
+                    <c:v>0.16329931618554538</c:v>
+                  </c:pt>
+                </c:numCache>
+              </c:numRef>
+            </c:minus>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:errBars>
+          <c:cat>
+            <c:strRef>
+              <c:f>Responstime!$U$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Mean Respons Time</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Responstime!$G$65</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>3.4</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-76BF-43A0-8D5B-5DBA4A6E9232}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Responstime!$H$63</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Pure</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:errBars>
+            <c:errBarType val="both"/>
+            <c:errValType val="cust"/>
+            <c:noEndCap val="0"/>
+            <c:plus>
+              <c:numRef>
+                <c:f>Responstime!$I$66</c:f>
+                <c:numCache>
+                  <c:formatCode>General</c:formatCode>
+                  <c:ptCount val="1"/>
+                  <c:pt idx="0">
+                    <c:v>9.9999999999999992E-2</c:v>
+                  </c:pt>
+                </c:numCache>
+              </c:numRef>
+            </c:plus>
+            <c:minus>
+              <c:numRef>
+                <c:f>Responstime!$I$66</c:f>
+                <c:numCache>
+                  <c:formatCode>General</c:formatCode>
+                  <c:ptCount val="1"/>
+                  <c:pt idx="0">
+                    <c:v>9.9999999999999992E-2</c:v>
+                  </c:pt>
+                </c:numCache>
+              </c:numRef>
+            </c:minus>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:errBars>
+          <c:cat>
+            <c:strRef>
+              <c:f>Responstime!$U$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Mean Respons Time</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Responstime!$I$65</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>3.1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-76BF-43A0-8D5B-5DBA4A6E9232}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1087486063"/>
+        <c:axId val="1087502863"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1087486063"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="sv-SE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1087502863"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1087502863"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="4.5"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="sv-SE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1087486063"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="sv-SE"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr baseline="0"/>
+      </a:pPr>
+      <a:endParaRPr lang="sv-SE"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -1103,6 +2166,86 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
@@ -1607,6 +2750,1012 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2178,6 +4327,78 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>4762</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>323850</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>80962</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B947D6C7-8101-CCDC-DCF1-370475421294}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>62</xdr:row>
+      <xdr:rowOff>23812</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>100012</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{34360E4A-1E21-30A7-B2B7-77646C4BC6B9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2503,12 +4724,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68065102-B80F-4809-BEA1-03E82A52692C}">
-  <dimension ref="A1:U36"/>
+  <dimension ref="A1:U77"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:21" ht="24" x14ac:dyDescent="0.4">
-      <c r="N1" s="4" t="s">
-        <v>16</v>
+      <c r="N1" s="3" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2529,16 +4750,16 @@
       <c r="C3">
         <v>11</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3" t="s">
+      <c r="G3" s="2"/>
+      <c r="H3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I3" s="3"/>
+      <c r="I3" s="2"/>
       <c r="U3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
@@ -2551,10 +4772,6 @@
       <c r="C4">
         <v>11</v>
       </c>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5">
@@ -2566,16 +4783,16 @@
       <c r="C5">
         <v>11</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" t="s">
         <v>0</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G5">
         <v>11</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" t="s">
         <v>0</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5">
         <v>10.666666666666666</v>
       </c>
     </row>
@@ -2589,16 +4806,16 @@
       <c r="C6">
         <v>11</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" t="s">
         <v>1</v>
       </c>
-      <c r="G6" s="1">
+      <c r="G6">
         <v>0.16666666666666666</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" t="s">
         <v>1</v>
       </c>
-      <c r="I6" s="1">
+      <c r="I6">
         <v>0.16666666666666666</v>
       </c>
     </row>
@@ -2612,16 +4829,16 @@
       <c r="C7">
         <v>10</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" t="s">
         <v>2</v>
       </c>
-      <c r="G7" s="1">
+      <c r="G7">
         <v>11</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="H7" t="s">
         <v>2</v>
       </c>
-      <c r="I7" s="1">
+      <c r="I7">
         <v>11</v>
       </c>
     </row>
@@ -2635,16 +4852,16 @@
       <c r="C8">
         <v>11</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" t="s">
         <v>3</v>
       </c>
-      <c r="G8" s="1">
+      <c r="G8">
         <v>11</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="H8" t="s">
         <v>3</v>
       </c>
-      <c r="I8" s="1">
+      <c r="I8">
         <v>11</v>
       </c>
     </row>
@@ -2658,16 +4875,16 @@
       <c r="C9">
         <v>10</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F9" t="s">
         <v>4</v>
       </c>
-      <c r="G9" s="1">
+      <c r="G9">
         <v>0.5</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="H9" t="s">
         <v>4</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I9">
         <v>0.5</v>
       </c>
     </row>
@@ -2681,16 +4898,16 @@
       <c r="C10">
         <v>10</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" t="s">
         <v>5</v>
       </c>
-      <c r="G10" s="1">
+      <c r="G10">
         <v>0.25</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="H10" t="s">
         <v>5</v>
       </c>
-      <c r="I10" s="1">
+      <c r="I10">
         <v>0.25000000000000006</v>
       </c>
     </row>
@@ -2704,106 +4921,106 @@
       <c r="C11">
         <v>11</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" t="s">
         <v>6</v>
       </c>
-      <c r="G11" s="1">
+      <c r="G11">
         <v>4</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="H11" t="s">
         <v>6</v>
       </c>
-      <c r="I11" s="1">
+      <c r="I11">
         <v>-1.7142857142857211</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="F12" s="1" t="s">
+      <c r="F12" t="s">
         <v>7</v>
       </c>
-      <c r="G12" s="1">
+      <c r="G12">
         <v>0</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="H12" t="s">
         <v>7</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I12">
         <v>-0.85714285714285277</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="F13" s="1" t="s">
+      <c r="F13" t="s">
         <v>8</v>
       </c>
-      <c r="G13" s="1">
+      <c r="G13">
         <v>2</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="H13" t="s">
         <v>8</v>
       </c>
-      <c r="I13" s="1">
+      <c r="I13">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="F14" s="1" t="s">
+      <c r="F14" t="s">
         <v>9</v>
       </c>
-      <c r="G14" s="1">
+      <c r="G14">
         <v>10</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="H14" t="s">
         <v>9</v>
       </c>
-      <c r="I14" s="1">
+      <c r="I14">
         <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="F15" s="1" t="s">
+      <c r="F15" t="s">
         <v>10</v>
       </c>
-      <c r="G15" s="1">
+      <c r="G15">
         <v>12</v>
       </c>
-      <c r="H15" s="1" t="s">
+      <c r="H15" t="s">
         <v>10</v>
       </c>
-      <c r="I15" s="1">
+      <c r="I15">
         <v>11</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="F16" s="1" t="s">
+      <c r="F16" t="s">
         <v>11</v>
       </c>
-      <c r="G16" s="1">
+      <c r="G16">
         <v>99</v>
       </c>
-      <c r="H16" s="1" t="s">
+      <c r="H16" t="s">
         <v>11</v>
       </c>
-      <c r="I16" s="1">
+      <c r="I16">
         <v>96</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F17" s="2" t="s">
+      <c r="F17" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G17" s="2">
+      <c r="G17" s="1">
         <v>9</v>
       </c>
-      <c r="H17" s="2" t="s">
+      <c r="H17" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17" s="1">
         <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="24" x14ac:dyDescent="0.4">
-      <c r="N20" s="4" t="s">
-        <v>15</v>
+      <c r="N20" s="3" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2824,14 +5041,14 @@
       <c r="C22">
         <v>11</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="F22" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3" t="s">
+      <c r="G22" s="2"/>
+      <c r="H22" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I22" s="3"/>
+      <c r="I22" s="2"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23">
@@ -2843,10 +5060,6 @@
       <c r="C23">
         <v>11</v>
       </c>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24">
@@ -2858,16 +5071,16 @@
       <c r="C24">
         <v>11</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="F24" t="s">
         <v>0</v>
       </c>
-      <c r="G24" s="1">
+      <c r="G24">
         <v>12.2</v>
       </c>
-      <c r="H24" s="1" t="s">
+      <c r="H24" t="s">
         <v>0</v>
       </c>
-      <c r="I24" s="1">
+      <c r="I24">
         <v>10.9</v>
       </c>
     </row>
@@ -2881,16 +5094,16 @@
       <c r="C25">
         <v>11</v>
       </c>
-      <c r="F25" s="1" t="s">
+      <c r="F25" t="s">
         <v>1</v>
       </c>
-      <c r="G25" s="1">
+      <c r="G25">
         <v>0.24944382578492943</v>
       </c>
-      <c r="H25" s="1" t="s">
+      <c r="H25" t="s">
         <v>1</v>
       </c>
-      <c r="I25" s="1">
+      <c r="I25">
         <v>9.9999999999999992E-2</v>
       </c>
     </row>
@@ -2904,16 +5117,16 @@
       <c r="C26">
         <v>11</v>
       </c>
-      <c r="F26" s="1" t="s">
+      <c r="F26" t="s">
         <v>2</v>
       </c>
-      <c r="G26" s="1">
+      <c r="G26">
         <v>12</v>
       </c>
-      <c r="H26" s="1" t="s">
+      <c r="H26" t="s">
         <v>2</v>
       </c>
-      <c r="I26" s="1">
+      <c r="I26">
         <v>11</v>
       </c>
     </row>
@@ -2927,16 +5140,16 @@
       <c r="C27">
         <v>11</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="F27" t="s">
         <v>3</v>
       </c>
-      <c r="G27" s="1">
+      <c r="G27">
         <v>13</v>
       </c>
-      <c r="H27" s="1" t="s">
+      <c r="H27" t="s">
         <v>3</v>
       </c>
-      <c r="I27" s="1">
+      <c r="I27">
         <v>11</v>
       </c>
     </row>
@@ -2950,16 +5163,16 @@
       <c r="C28">
         <v>11</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="F28" t="s">
         <v>4</v>
       </c>
-      <c r="G28" s="1">
+      <c r="G28">
         <v>0.78881063774661553</v>
       </c>
-      <c r="H28" s="1" t="s">
+      <c r="H28" t="s">
         <v>4</v>
       </c>
-      <c r="I28" s="1">
+      <c r="I28">
         <v>0.31622776601683794</v>
       </c>
     </row>
@@ -2973,16 +5186,16 @@
       <c r="C29">
         <v>11</v>
       </c>
-      <c r="F29" s="1" t="s">
+      <c r="F29" t="s">
         <v>5</v>
       </c>
-      <c r="G29" s="1">
+      <c r="G29">
         <v>0.62222222222222234</v>
       </c>
-      <c r="H29" s="1" t="s">
+      <c r="H29" t="s">
         <v>5</v>
       </c>
-      <c r="I29" s="1">
+      <c r="I29">
         <v>9.9999999999999992E-2</v>
       </c>
     </row>
@@ -2996,16 +5209,16 @@
       <c r="C30">
         <v>10</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="F30" t="s">
         <v>6</v>
       </c>
-      <c r="G30" s="1">
+      <c r="G30">
         <v>-1.0741618075801784</v>
       </c>
-      <c r="H30" s="1" t="s">
+      <c r="H30" t="s">
         <v>6</v>
       </c>
-      <c r="I30" s="1">
+      <c r="I30">
         <v>10.000000000000018</v>
       </c>
     </row>
@@ -3019,86 +5232,688 @@
       <c r="C31">
         <v>11</v>
       </c>
-      <c r="F31" s="1" t="s">
+      <c r="F31" t="s">
         <v>7</v>
       </c>
-      <c r="G31" s="1">
+      <c r="G31">
         <v>-0.40748508710124526</v>
       </c>
-      <c r="H31" s="1" t="s">
+      <c r="H31" t="s">
         <v>7</v>
       </c>
-      <c r="I31" s="1">
+      <c r="I31">
         <v>-3.1622776601683831</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F32" s="1" t="s">
+      <c r="F32" t="s">
         <v>8</v>
       </c>
-      <c r="G32" s="1">
+      <c r="G32">
         <v>2</v>
       </c>
-      <c r="H32" s="1" t="s">
+      <c r="H32" t="s">
         <v>8</v>
       </c>
-      <c r="I32" s="1">
+      <c r="I32">
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="6:9" x14ac:dyDescent="0.25">
-      <c r="F33" s="1" t="s">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F33" t="s">
         <v>9</v>
       </c>
-      <c r="G33" s="1">
+      <c r="G33">
         <v>11</v>
       </c>
-      <c r="H33" s="1" t="s">
+      <c r="H33" t="s">
         <v>9</v>
       </c>
-      <c r="I33" s="1">
+      <c r="I33">
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="6:9" x14ac:dyDescent="0.25">
-      <c r="F34" s="1" t="s">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F34" t="s">
         <v>10</v>
       </c>
-      <c r="G34" s="1">
+      <c r="G34">
         <v>13</v>
       </c>
-      <c r="H34" s="1" t="s">
+      <c r="H34" t="s">
         <v>10</v>
       </c>
-      <c r="I34" s="1">
+      <c r="I34">
         <v>11</v>
       </c>
     </row>
-    <row r="35" spans="6:9" x14ac:dyDescent="0.25">
-      <c r="F35" s="1" t="s">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F35" t="s">
         <v>11</v>
       </c>
-      <c r="G35" s="1">
+      <c r="G35">
         <v>122</v>
       </c>
-      <c r="H35" s="1" t="s">
+      <c r="H35" t="s">
         <v>11</v>
       </c>
-      <c r="I35" s="1">
+      <c r="I35">
         <v>109</v>
       </c>
     </row>
-    <row r="36" spans="6:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F36" s="2" t="s">
+    <row r="36" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F36" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G36" s="2">
+      <c r="G36" s="1">
         <v>10</v>
       </c>
-      <c r="H36" s="2" t="s">
+      <c r="H36" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I36" s="2">
+      <c r="I36" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="24" x14ac:dyDescent="0.4">
+      <c r="N40" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B42" t="s">
+        <v>13</v>
+      </c>
+      <c r="C42" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>1</v>
+      </c>
+      <c r="B43">
+        <v>4</v>
+      </c>
+      <c r="C43">
+        <v>3</v>
+      </c>
+      <c r="F43" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G43" s="6"/>
+      <c r="H43" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="I43" s="6"/>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>2</v>
+      </c>
+      <c r="B44">
+        <v>5</v>
+      </c>
+      <c r="C44">
+        <v>3</v>
+      </c>
+      <c r="F44" s="4"/>
+      <c r="G44" s="4"/>
+      <c r="H44" s="4"/>
+      <c r="I44" s="4"/>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>3</v>
+      </c>
+      <c r="B45">
+        <v>4</v>
+      </c>
+      <c r="C45">
+        <v>3</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="G45" s="4">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="I45" s="4">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>4</v>
+      </c>
+      <c r="B46">
+        <v>4</v>
+      </c>
+      <c r="C46">
+        <v>3</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G46" s="4">
+        <v>0.17950549357115031</v>
+      </c>
+      <c r="H46" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I46" s="4">
+        <v>9.9999999999999992E-2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>5</v>
+      </c>
+      <c r="B47">
+        <v>4</v>
+      </c>
+      <c r="C47">
+        <v>3</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="G47" s="4">
+        <v>4</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="I47" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>6</v>
+      </c>
+      <c r="B48">
+        <v>4</v>
+      </c>
+      <c r="C48">
+        <v>3</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="G48" s="4">
+        <v>4</v>
+      </c>
+      <c r="H48" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="I48" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>7</v>
+      </c>
+      <c r="B49">
+        <v>4</v>
+      </c>
+      <c r="C49">
+        <v>3</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G49" s="4">
+        <v>0.5676462121975473</v>
+      </c>
+      <c r="H49" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="I49" s="4">
+        <v>0.31622776601683794</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>8</v>
+      </c>
+      <c r="B50">
+        <v>4</v>
+      </c>
+      <c r="C50">
+        <v>4</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G50" s="4">
+        <v>0.32222222222222285</v>
+      </c>
+      <c r="H50" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I50" s="4">
+        <v>9.9999999999999992E-2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>9</v>
+      </c>
+      <c r="B51">
+        <v>5</v>
+      </c>
+      <c r="C51">
+        <v>3</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G51" s="4">
+        <v>1.4982164090368641</v>
+      </c>
+      <c r="H51" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I51" s="4">
+        <v>9.9999999999999929</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>10</v>
+      </c>
+      <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52">
+        <v>3</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G52" s="4">
+        <v>9.1120378890214848E-2</v>
+      </c>
+      <c r="H52" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I52" s="4">
+        <v>3.1622776601683782</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F53" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G53" s="4">
+        <v>2</v>
+      </c>
+      <c r="H53" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I53" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F54" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G54" s="4">
+        <v>3</v>
+      </c>
+      <c r="H54" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="I54" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F55" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G55" s="4">
+        <v>5</v>
+      </c>
+      <c r="H55" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I55" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F56" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G56" s="4">
+        <v>41</v>
+      </c>
+      <c r="H56" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I56" s="4">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F57" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G57" s="5">
+        <v>10</v>
+      </c>
+      <c r="H57" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I57" s="5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" ht="24" x14ac:dyDescent="0.4">
+      <c r="N60" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B62" t="s">
+        <v>13</v>
+      </c>
+      <c r="C62" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>1</v>
+      </c>
+      <c r="B63">
+        <v>4</v>
+      </c>
+      <c r="C63">
+        <v>4</v>
+      </c>
+      <c r="F63" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G63" s="6"/>
+      <c r="H63" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="I63" s="6"/>
+    </row>
+    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>2</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64">
+        <v>3</v>
+      </c>
+      <c r="F64" s="4"/>
+      <c r="G64" s="4"/>
+      <c r="H64" s="4"/>
+      <c r="I64" s="4"/>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>3</v>
+      </c>
+      <c r="B65">
+        <v>4</v>
+      </c>
+      <c r="C65">
+        <v>3</v>
+      </c>
+      <c r="F65" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="G65" s="4">
+        <v>3.4</v>
+      </c>
+      <c r="H65" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="I65" s="4">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>4</v>
+      </c>
+      <c r="B66">
+        <v>3</v>
+      </c>
+      <c r="C66">
+        <v>3</v>
+      </c>
+      <c r="F66" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G66" s="4">
+        <v>0.16329931618554538</v>
+      </c>
+      <c r="H66" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I66" s="4">
+        <v>9.9999999999999992E-2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>5</v>
+      </c>
+      <c r="B67">
+        <v>4</v>
+      </c>
+      <c r="C67">
+        <v>3</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="G67" s="4">
+        <v>3</v>
+      </c>
+      <c r="H67" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="I67" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>6</v>
+      </c>
+      <c r="B68">
+        <v>3</v>
+      </c>
+      <c r="C68">
+        <v>3</v>
+      </c>
+      <c r="F68" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="G68" s="4">
+        <v>3</v>
+      </c>
+      <c r="H68" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="I68" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>7</v>
+      </c>
+      <c r="B69">
+        <v>3</v>
+      </c>
+      <c r="C69">
+        <v>3</v>
+      </c>
+      <c r="F69" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G69" s="4">
+        <v>0.51639777949432286</v>
+      </c>
+      <c r="H69" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="I69" s="4">
+        <v>0.31622776601683794</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>8</v>
+      </c>
+      <c r="B70">
+        <v>3</v>
+      </c>
+      <c r="C70">
+        <v>3</v>
+      </c>
+      <c r="F70" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G70" s="4">
+        <v>0.26666666666666727</v>
+      </c>
+      <c r="H70" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I70" s="4">
+        <v>9.9999999999999992E-2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>9</v>
+      </c>
+      <c r="B71">
+        <v>4</v>
+      </c>
+      <c r="C71">
+        <v>3</v>
+      </c>
+      <c r="F71" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G71" s="4">
+        <v>-2.2767857142857149</v>
+      </c>
+      <c r="H71" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I71" s="4">
+        <v>10.000000000000004</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>10</v>
+      </c>
+      <c r="B72">
+        <v>3</v>
+      </c>
+      <c r="C72">
+        <v>3</v>
+      </c>
+      <c r="F72" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G72" s="4">
+        <v>0.48412291827592785</v>
+      </c>
+      <c r="H72" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I72" s="4">
+        <v>3.1622776601683791</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F73" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G73" s="4">
+        <v>1</v>
+      </c>
+      <c r="H73" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I73" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F74" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G74" s="4">
+        <v>3</v>
+      </c>
+      <c r="H74" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="I74" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F75" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G75" s="4">
+        <v>4</v>
+      </c>
+      <c r="H75" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="I75" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F76" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G76" s="4">
+        <v>34</v>
+      </c>
+      <c r="H76" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I76" s="4">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F77" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G77" s="5">
+        <v>10</v>
+      </c>
+      <c r="H77" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I77" s="5">
         <v>10</v>
       </c>
     </row>

</xml_diff>